<commit_message>
bs pendiente por debbugear
</commit_message>
<xml_diff>
--- a/data/Mina_modelo_costo_fijo_BS/elmo_data.xlsx
+++ b/data/Mina_modelo_costo_fijo_BS/elmo_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\Elmo_infrastructure_NP\data\Mina_modelo_costo_fijo_BS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22FFBB25-F49C-4042-9134-F86050E4F40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92B57914-0EF2-4D6A-A2C8-4756B8E24314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2248,8 +2248,7 @@
         <v>8.3000000000000004E-2</v>
       </c>
       <c r="AE3">
-        <f>($Z$3-$Z$3*$AA$3)/chargers!$D$3</f>
-        <v>0.79999999999999993</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:31" ht="23.7" customHeight="1" x14ac:dyDescent="0.3">
@@ -2344,8 +2343,7 @@
         <v>8.3000000000000004E-2</v>
       </c>
       <c r="AE4">
-        <f>($Z$3-$Z$3*$AA$3)/chargers!$D$3</f>
-        <v>0.79999999999999993</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:31" ht="23.7" customHeight="1" x14ac:dyDescent="0.3">
@@ -2440,8 +2438,7 @@
         <v>8.3000000000000004E-2</v>
       </c>
       <c r="AE5">
-        <f>($Z$3-$Z$3*$AA$3)/chargers!$D$3</f>
-        <v>0.79999999999999993</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:31" ht="23.7" customHeight="1" x14ac:dyDescent="0.3">
@@ -2536,8 +2533,8 @@
         <v>8.3000000000000004E-2</v>
       </c>
       <c r="AE6">
-        <f>($Z$3-$Z$3*$AA$3)/chargers!$D$3</f>
-        <v>0.79999999999999993</v>
+        <f>AE3</f>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:31" ht="23.7" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>